<commit_message>
sua file data test lan 2
</commit_message>
<xml_diff>
--- a/DahlaFlowerShop/test/AutomationFramework/testdata/test_data.xlsx
+++ b/DahlaFlowerShop/test/AutomationFramework/testdata/test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T14s-Gen1\Desktop\DATN\DahlaFlowerShop\test\AutomationFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB6C5CC-36C8-4EE2-B1EC-CD1D511D5AD7}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B4B0B8-7BFC-4E09-A442-643323E189D6}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="330">
   <si>
     <t>id</t>
   </si>
@@ -540,9 +540,6 @@
     <t>Username chứa ký tự đặc biệt</t>
   </si>
   <si>
-    <t>adm!n</t>
-  </si>
-  <si>
     <t>L17</t>
   </si>
   <si>
@@ -558,12 +555,6 @@
     <t>L19</t>
   </si>
   <si>
-    <t>Username quá dài</t>
-  </si>
-  <si>
-    <t>adminadminadminadmin</t>
-  </si>
-  <si>
     <t>L20</t>
   </si>
   <si>
@@ -585,12 +576,6 @@
     <t>L22</t>
   </si>
   <si>
-    <t>Username có dấu tiếng Việt</t>
-  </si>
-  <si>
-    <t>admín</t>
-  </si>
-  <si>
     <t>L23</t>
   </si>
   <si>
@@ -639,103 +624,28 @@
     <t>L28</t>
   </si>
   <si>
-    <t>Username null</t>
-  </si>
-  <si>
-    <t>null</t>
-  </si>
-  <si>
-    <t>L29</t>
-  </si>
-  <si>
-    <t>Password null</t>
-  </si>
-  <si>
-    <t>L30</t>
-  </si>
-  <si>
-    <t>Username và password null</t>
-  </si>
-  <si>
-    <t>L31</t>
-  </si>
-  <si>
-    <t>Username chứa emoji</t>
-  </si>
-  <si>
-    <t>admin😀</t>
-  </si>
-  <si>
-    <t>L32</t>
-  </si>
-  <si>
-    <t>Password chứa emoji</t>
-  </si>
-  <si>
-    <t>pass😀123</t>
-  </si>
-  <si>
-    <t>L33</t>
-  </si>
-  <si>
-    <t>Username chỉ chứa khoảng trắng</t>
-  </si>
-  <si>
-    <t>" "</t>
-  </si>
-  <si>
-    <t>L34</t>
-  </si>
-  <si>
-    <t>Password chỉ chứa khoảng trắng</t>
-  </si>
-  <si>
-    <t>L35</t>
-  </si>
-  <si>
     <t>Username có tab</t>
   </si>
   <si>
     <t>admin\t</t>
   </si>
   <si>
-    <t>L36</t>
-  </si>
-  <si>
     <t>Password có tab</t>
   </si>
   <si>
     <t>123\t</t>
   </si>
   <si>
-    <t>L37</t>
-  </si>
-  <si>
     <t>Username có xuống dòng</t>
   </si>
   <si>
     <t>admin\n</t>
   </si>
   <si>
-    <t>L38</t>
-  </si>
-  <si>
     <t>Password có xuống dòng</t>
   </si>
   <si>
     <t>123\n</t>
-  </si>
-  <si>
-    <t>L39</t>
-  </si>
-  <si>
-    <t>Ký tự Unicode trong username</t>
-  </si>
-  <si>
-    <t>用户名</t>
-  </si>
-  <si>
-    <t>L40</t>
   </si>
   <si>
     <t>Ký tự Unicode trong password</t>
@@ -1512,7 +1422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1667,7 +1577,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>154</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1684,7 +1594,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>157</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -1701,7 +1611,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>160</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1718,7 +1628,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>162</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -1735,7 +1645,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>164</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1752,7 +1662,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>166</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -1769,7 +1679,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>168</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -1786,427 +1696,223 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>170</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1.23456789012345E+19</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D17" s="4">
+      <c r="B18" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D18" s="4">
         <v>123</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="E18" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="4">
-        <v>1</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>175</v>
-      </c>
       <c r="B19" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="4">
-        <v>1.23456789012345E+19</v>
+      <c r="D19" s="4" t="s">
+        <v>182</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="D20" s="4">
-        <v>123</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>180</v>
-      </c>
       <c r="B21" s="4" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="D21" s="4">
         <v>123</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>183</v>
+      <c r="A22" s="5" t="s">
+        <v>180</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>186</v>
+      <c r="A23" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D23" s="4">
         <v>123</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>12</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>189</v>
+      <c r="A24" s="5" t="s">
+        <v>184</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
-        <v>192</v>
+      <c r="A25" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="D25" s="4">
         <v>123</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>196</v>
+      <c r="A26" s="5" t="s">
+        <v>191</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>198</v>
+      <c r="A27" s="5" t="s">
+        <v>193</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D27" s="4">
         <v>123</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>201</v>
+      <c r="A28" s="5" t="s">
+        <v>196</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>204</v>
+      <c r="A29" s="5" t="s">
+        <v>199</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="D29" s="4">
-        <v>123</v>
+        <v>7</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>209</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="D32" s="4">
-        <v>123</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="D34" s="4">
-        <v>123</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="D36" s="4">
-        <v>123</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="D38" s="4">
-        <v>123</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="D40" s="4">
-        <v>123</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="E41" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2519,10 +2225,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>7</v>
@@ -2531,10 +2237,10 @@
         <v>40</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>242</v>
+        <v>212</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="G10" s="6">
         <v>912345678</v>
@@ -2549,18 +2255,18 @@
         <v>46</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>246</v>
+        <v>216</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>40</v>
@@ -2569,7 +2275,7 @@
         <v>41</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>248</v>
+        <v>218</v>
       </c>
       <c r="G11" s="6">
         <v>912345679</v>
@@ -2578,33 +2284,33 @@
         <v>35866</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>46</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>250</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>251</v>
+        <v>221</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="D12" s="6">
         <v>123</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>253</v>
+        <v>223</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>254</v>
+        <v>224</v>
       </c>
       <c r="G12" s="6">
         <v>987654321</v>
@@ -2613,7 +2319,7 @@
         <v>37143</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>255</v>
+        <v>225</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>46</v>
@@ -2624,22 +2330,22 @@
     </row>
     <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>256</v>
+        <v>226</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>257</v>
+        <v>227</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>258</v>
+        <v>228</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>259</v>
+        <v>229</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>260</v>
+        <v>230</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>261</v>
+        <v>231</v>
       </c>
       <c r="G13" s="6">
         <v>987123456</v>
@@ -2654,27 +2360,27 @@
         <v>56</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>264</v>
+        <v>234</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>265</v>
+        <v>235</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>266</v>
+        <v>236</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>267</v>
+        <v>237</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>268</v>
+        <v>238</v>
       </c>
       <c r="G14" s="6">
         <v>911111111</v>
@@ -2689,27 +2395,27 @@
         <v>46</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>269</v>
+        <v>239</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>270</v>
+        <v>240</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>271</v>
+        <v>241</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>272</v>
+        <v>242</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>273</v>
+        <v>243</v>
       </c>
       <c r="G15" s="6">
         <v>922222222</v>
@@ -2718,7 +2424,7 @@
         <v>35285</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>274</v>
+        <v>244</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>46</v>
@@ -2729,22 +2435,22 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>275</v>
+        <v>245</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>276</v>
+        <v>246</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>277</v>
+        <v>247</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>278</v>
+        <v>248</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>279</v>
+        <v>249</v>
       </c>
       <c r="G16" s="6">
         <v>933333333</v>
@@ -2753,7 +2459,7 @@
         <v>34803</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>56</v>
@@ -2764,31 +2470,31 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>281</v>
+        <v>251</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>282</v>
+        <v>252</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>283</v>
+        <v>253</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>284</v>
+        <v>254</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>285</v>
+        <v>255</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>286</v>
+        <v>256</v>
       </c>
       <c r="H17" s="8">
         <v>37539</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>287</v>
+        <v>257</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>46</v>
@@ -2799,22 +2505,22 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>288</v>
+        <v>258</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>289</v>
+        <v>259</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>290</v>
+        <v>260</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>291</v>
+        <v>261</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>292</v>
+        <v>262</v>
       </c>
       <c r="G18" s="6">
         <v>9876</v>
@@ -2823,7 +2529,7 @@
         <v>37622</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>293</v>
+        <v>263</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>56</v>
@@ -2834,22 +2540,22 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>294</v>
+        <v>264</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>295</v>
+        <v>265</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>296</v>
+        <v>266</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>297</v>
+        <v>267</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>298</v>
+        <v>268</v>
       </c>
       <c r="G19" s="6">
         <v>123456789123</v>
@@ -2869,22 +2575,22 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>299</v>
+        <v>269</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>301</v>
+        <v>271</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>302</v>
+        <v>272</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>303</v>
+        <v>273</v>
       </c>
       <c r="G20" s="6">
         <v>977777777</v>
@@ -2893,33 +2599,33 @@
         <v>35952</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>46</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>304</v>
+        <v>274</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>171</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>305</v>
+        <v>275</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>306</v>
+        <v>276</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>307</v>
+        <v>277</v>
       </c>
       <c r="G21" s="6">
         <v>966666666</v>
@@ -2934,27 +2640,27 @@
         <v>46</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>308</v>
+        <v>278</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>309</v>
+        <v>279</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>310</v>
+        <v>280</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>311</v>
+        <v>281</v>
       </c>
       <c r="G22" s="6">
         <v>955555555</v>
@@ -2969,27 +2675,27 @@
         <v>46</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>312</v>
+        <v>282</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>313</v>
+        <v>283</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>314</v>
+        <v>284</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>315</v>
+        <v>285</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>316</v>
+        <v>286</v>
       </c>
       <c r="G23" s="6">
         <v>944444444</v>
@@ -2998,33 +2704,33 @@
         <v>36175</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>274</v>
+        <v>244</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>46</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
-        <v>317</v>
+        <v>287</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>319</v>
+        <v>289</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>321</v>
+        <v>291</v>
       </c>
       <c r="G24" s="6">
         <v>933333334</v>
@@ -3042,22 +2748,22 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>322</v>
+        <v>292</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>323</v>
+        <v>293</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>324</v>
+        <v>294</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>325</v>
+        <v>295</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>326</v>
+        <v>296</v>
       </c>
       <c r="G25" s="6">
         <v>922222223</v>
@@ -3072,27 +2778,27 @@
         <v>46</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>327</v>
+        <v>297</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>328</v>
+        <v>298</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>329</v>
+        <v>299</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>330</v>
+        <v>300</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>331</v>
+        <v>301</v>
       </c>
       <c r="G26" s="6">
         <v>911111112</v>
@@ -3110,22 +2816,22 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>332</v>
+        <v>302</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>333</v>
+        <v>303</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>334</v>
+        <v>304</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>335</v>
+        <v>305</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>336</v>
+        <v>306</v>
       </c>
       <c r="G27" s="6">
         <v>900000000</v>
@@ -3143,22 +2849,22 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
-        <v>337</v>
+        <v>307</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>155</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>338</v>
+        <v>308</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>339</v>
+        <v>309</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>340</v>
+        <v>310</v>
       </c>
       <c r="G28" s="6">
         <v>988888888</v>
@@ -3167,7 +2873,7 @@
         <v>33436</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>46</v>
@@ -3178,22 +2884,22 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>341</v>
+        <v>311</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>342</v>
+        <v>312</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>343</v>
+        <v>313</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>344</v>
+        <v>314</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>345</v>
+        <v>315</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>346</v>
+        <v>316</v>
       </c>
       <c r="G29" s="6">
         <v>971234567</v>
@@ -3202,33 +2908,33 @@
         <v>36121</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>347</v>
+        <v>317</v>
       </c>
       <c r="J29" s="6" t="s">
         <v>56</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>348</v>
+        <v>318</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>349</v>
+        <v>319</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>350</v>
+        <v>320</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>351</v>
+        <v>321</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>352</v>
+        <v>322</v>
       </c>
       <c r="G30" s="6">
         <v>962345678</v>
@@ -3248,22 +2954,22 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>353</v>
+        <v>323</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>354</v>
+        <v>324</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>355</v>
+        <v>325</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>356</v>
+        <v>326</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>357</v>
+        <v>327</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>358</v>
+        <v>328</v>
       </c>
       <c r="G31" s="6">
         <v>912340000</v>
@@ -3272,7 +2978,7 @@
         <v>36412</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>359</v>
+        <v>329</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>56</v>

</xml_diff>